<commit_message>
daily: update content research log
</commit_message>
<xml_diff>
--- a/content_log.xlsx
+++ b/content_log.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O50"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3128,6 +3128,1066 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>AI artificial intelligence</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence for Automated Analysis and Interpretation of Intravascular Ultrasound in Coronary Artery Disease: A Systematic Review - Cureus</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>Cureus</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipAJBVV95cUxQRGU5cGhYWUY3NDNtaURrcmpqZTRDN3ZHQlk1ZHV2UUVvbEI5S2ZDM3BOaUR4N3Q0LXYwcjh3cTh6WnFkdnBhY2xtTjJ6OWdCeHVScHZOTXdPa0RjNkVzWkVtMTU0aFBGQWVMSmVRdVZva0UzVTU0SExaUGJicGFfQU00WjZEdG5FUWhMRnFHdnF5VHI2Smc0R0tvQjFTRFQtWDR0TUJuN20tYTJRbnFzRUNlTmNJT0FWc0xhX3FYaFUwRWM5STZGbktRcTlobkh1NTlOMlNMQl9xS1lwU0syZUpxeXMwdGNzd0VpSGlWNlpiX0h2RnVkUmtiVzVhVkVBQ19LdTc2QlhjcVJtVHY2bWpzdU9MRkZBZTBLQzFWTnc4VUJK?oc=5</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T11:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="n"/>
+      <c r="I51" s="2" t="n"/>
+      <c r="J51" s="2" t="n"/>
+      <c r="K51" s="2" t="n"/>
+      <c r="L51" s="2" t="n"/>
+      <c r="M51" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>AI artificial intelligence</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI safety employee quits, warns AI firms aren't doing enough on risks - Business Standard</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>Business Standard</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi8wFBVV95cUxPTkJlQzBLV2d4RTdmSXlhT0lUV1hBYm53a2NxT2xJck9oaURZYjNsMWptM21YTGUzeHN5RkNFUlpzclNrUUh4Zjk0b0tWTGxmdWp0NHo4cWhVUWVmZVAzMVRLcGkwNG8yeGo3Ym5Sd05sdWQ2aVg3eG10MExxTmU5TVBsdlM2Z2ZaOVl2dUNVdlBxMENBYU9GQjNkVGc5b3ljdDV5cnBWZFdJYW5rS0dMSTNPV0R2YkZiRTdaUHlFeWdBS3Njcl94NnNyYjFxaHJZMFN2dXBDX05wcjJaSXAtVWpnbi16YlRvelo3bWt1YlprNGvSAfgBQVVfeXFMTkg2aGluakVaU1VWdXVkamtXaG53dVdLZEtOMHExWkVValNRZEJucVpSVnAzakJPeVFLdXJkU3R0MjhBSmk0c2FGVlBhdG9PVTgwSTFPeks3SWtTT3I3bjZDN1Z4MkNRN2w4dlA4MG9nRGotWF9YMjhHbkVtcWtvNzhPZ3RzQjJUOEY1NDZLWFlmUHVZYkJJMXZBSl95cEZqWWZkWWNnb3pTdEtHOTBFRjRPTjlmUkhiTkpyWTVLRHJ5bDJKY2lDRGpkQmpRUm83dVVnc1hMVlBOZkJ2b2dKNDVXUGdJR01zUlUxWnQ1QV9JbWhVOERPRGI?oc=5</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:52:38+00:00</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="n"/>
+      <c r="I52" s="2" t="n"/>
+      <c r="J52" s="2" t="n"/>
+      <c r="K52" s="2" t="n"/>
+      <c r="L52" s="2" t="n"/>
+      <c r="M52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>I Quit OpenAI Because Its Culture Is Broken - The Atlantic</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>The Atlantic</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPX2NNSzBoT3NhRmFhWjdUZ1NtOTFVNUFRaFBvNUd2R1c2NlhCLVZNanZfdm5UR3BDZ2V0bC1Oa00zano0OWtDdUo3WFFzMXNqdUxDczJ2Ujl3Vng5N2VlRGZDeWx5OHBhbWFnTXZpNkVTbWNHOFMtTEcyLXFGckl4bDRtUE81ZnIyWU91S21n?oc=5</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T11:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="n"/>
+      <c r="I53" s="2" t="n"/>
+      <c r="J53" s="2" t="n"/>
+      <c r="K53" s="2" t="n"/>
+      <c r="L53" s="2" t="n"/>
+      <c r="M53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N53" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O53" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI discloses another Australian government hack - Mashable</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Mashable</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiiAFBVV95cUxNQ1o1T2dBczJSZjhVTmlPcEljLWQzTTc0aVZLSUY4a1I3eF9ZSTBTYTZIb2g4bHpwU3pJSTBWUDZoc1RscUtYVWRfVkNFVS1VdnlZeG8yQ0tYbjZtVkxnOF9tT2EyWEFuNy0yVmZMM2NpekNzc0dWYmx4c1F2ZkVIbldlSFpTQUJG?oc=5</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T09:06:05+00:00</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="n"/>
+      <c r="I54" s="2" t="n"/>
+      <c r="J54" s="2" t="n"/>
+      <c r="K54" s="2" t="n"/>
+      <c r="L54" s="2" t="n"/>
+      <c r="M54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N54" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O54" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>Exclusive / How employees forced OpenAI’s president to back down - Semafor</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>Semafor</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMimgFBVV95cUxOQkNIaGItUndIa2RoYVZ4QVh1RE5XOUFkN2NrQUhqdjRfVS0yc2x4VzdaQWFraDVzeVFVcTF0amc4LTJfM2hyU0RwWkVKZERyS3lMLXo1V0pYSWVXUUFYc1RuX2h4aVp2UHZPMThNZkVzcG1ZbjROOXlxOHBDaDV6SGd1LVYyMm9JQkRuUmhnb0MwTVBSeV9mVWhR?oc=5</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T22:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="n"/>
+      <c r="I55" s="2" t="n"/>
+      <c r="J55" s="2" t="n"/>
+      <c r="K55" s="2" t="n"/>
+      <c r="L55" s="2" t="n"/>
+      <c r="M55" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N55" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O55" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>The eternal complement - OpenAI</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiXEFVX3lxTFBVWmpWcUY1SVAtVWc2bnhmNHhSOWVFYnY4aGR3RG4xRHZwWlNNdFhwRS1aSUZhQk5kNUpGRnhBdU03T01rU0JXaWdnQ1hPck1RT0lCbE03V3Q5Ti05?oc=5</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:41:33+00:00</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="n"/>
+      <c r="I56" s="2" t="n"/>
+      <c r="J56" s="2" t="n"/>
+      <c r="K56" s="2" t="n"/>
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="D57" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI says its review into hacks, including on Australian government sites, is costing $500,000 a day - The Guardian</t>
+        </is>
+      </c>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>The Guardian</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuwFBVV95cUxPQV9vbzIxazFuRjRrZVRqQnF1c2toZ1dMcnMxTUN4Uk5ISVNFQ1Q4aGdSd0t6aE16YjMzZ09nWGVHdUYzUE1jN0IyOThnYUNVTEdBNFlEWkJ1LVhBOU0yNGZwWnRvWGgwNTUyTTVNX1BnVkRvb2g1WFlmTDBTcGdfYUd2bGhHWFdycFY4WWFiSGxYOVR2QldpR3VnN0VsLW1JWDFBTUxlTFN6UTVwRjBVRGxjRlE3M3JSRnVV?oc=5</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T05:40:00+00:00</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="n"/>
+      <c r="I57" s="2" t="n"/>
+      <c r="J57" s="2" t="n"/>
+      <c r="K57" s="2" t="n"/>
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N57" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Google Gemini AI</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Google Wants AI Content Fact-Checked, Gemini UTM Tags – SEO Pulse - Search Engine Journal</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>Search Engine Journal</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMinwFBVV95cUxOcTZBQURKU0RqM0g1LTY5ZFdBU25OQzY2UmtYSEFGdDFmNXpOYnhmTWc5TjUtRndWNW9aVGZMY2JYazdXMHZTanZGWnZSU1VKZEZQNGxqZXkwcEZnNUNIVkRFNVJBbGtiNldVSEE1NGFSYzlWTWdkaUFQMnZoWDU0dUxPTjZzZ3BIdkU2Y1BiNWVqbXh0Wkc0VThIOExRakk?oc=5</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:00:26+00:00</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="n"/>
+      <c r="I58" s="2" t="n"/>
+      <c r="J58" s="2" t="n"/>
+      <c r="K58" s="2" t="n"/>
+      <c r="L58" s="2" t="n"/>
+      <c r="M58" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N58" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Google Gemini AI</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>Google Pushed AI Into Schools—and Even Students Say It’s Gone Too Far - WSJ</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>WSJ</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMie0FVX3lxTE1GQ1g3MkhsR1VXWmJvLXU2UDYyMVR5ekl6aFJPc21nZW9GZUN6S2JwQkJNdHFFbHMtS2E3MlFTNnEtWFpsZHhRX2lhWVBsTEpZbm5ENGZha0hqb3hoT21aT0hLQ1FrSHdXVWJMUXB6R0pFeXphTnZqQ05VRQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T16:31:56+00:00</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
+      <c r="M59" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N59" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Google Gemini AI</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Just days after Gemini Argon launch, Google updates AI plans to limit free use significantly - Neowin</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Neowin</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMivAFBVV95cUxQTnd0N3VMdHQ1aFJwUHZSVVdyaldycG5oXzZrRU1HTVZnWUpONUgtaEgyc2NyLTFPVERPRU5qZG4yYXZIcVRiMFJSOUdUd3RJRjc1Vk10NjhEZE1NMlg3bFE5aGZGUDloXzJuMXpnYngxR1RCSDVFNVoxQTJvZ2M2TXhWUGlqc1BfaHRIVmJwLWF3WmM5cTlHNGR0dVd4aHNlVDBfNW0zYkNrbHFxU2luQkxxQkZXSkxNUmN3UQ?oc=5</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T10:48:00+00:00</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="n"/>
+      <c r="I60" s="2" t="n"/>
+      <c r="J60" s="2" t="n"/>
+      <c r="K60" s="2" t="n"/>
+      <c r="L60" s="2" t="n"/>
+      <c r="M60" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N60" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Copilot AI</t>
+        </is>
+      </c>
+      <c r="D61" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft adds agent governance and usage controls to Copilot - msspalert.com</t>
+        </is>
+      </c>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>msspalert.com</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiowFBVV95cUxOM2o1X2tTWFdQRzNlYS0zdjFkUjZrcXhEUVItUXExUkJUdFhpNnlVbkxtcWMxS1dMTTNFNnYzVjFyYm5QeVBZY2pqRmxrY2dBcHhqMFctbVVsWWRCd2tab3hqUFZrbDd4czZwVE94WC1iMGNZdGhQWm9oYWRDSTlpQTEtLWxUZ3IxeU9COWJjcWZPb3hHYmJta1k4eUV6YWVmVmRJ?oc=5</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:00:00+00:00</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="n"/>
+      <c r="I61" s="2" t="n"/>
+      <c r="J61" s="2" t="n"/>
+      <c r="K61" s="2" t="n"/>
+      <c r="L61" s="2" t="n"/>
+      <c r="M61" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N61" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA AI</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>US arrests tech CEO accused of smuggling $300M in Nvidia chips into China - Ars Technica</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Ars Technica</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiuAFBVV95cUxPVlhTZzZkSkdEUlZRM1lhSlFCbTJvU1BPOVRmX0RGeGlkWGU2RTBCZzdOQWJsTDlFY1g4Q1pRRFA2aVlaSDItaVpUaC1zNURkUFh1TlBzS3VqQU91Q0NqV254NXphOG1OTEpWUTVwVzA1SXVWbzVYRHVfWlBSTXV2MzlxV0dFLTZzZ2VEQ1QtMDFBa2ozWmw0ZEphUWl6bnB3OXNLU3JWNFU3MzJwcV96VFJhTWVfQWNr?oc=5</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-02T18:39:36+00:00</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="n"/>
+      <c r="I62" s="2" t="n"/>
+      <c r="J62" s="2" t="n"/>
+      <c r="K62" s="2" t="n"/>
+      <c r="L62" s="2" t="n"/>
+      <c r="M62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>NVIDIA AI</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>Nvidia breaks to all-time high of $237.87, driven by buyback, analyst upgrade, and AI demand - Investing.com</t>
+        </is>
+      </c>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>Investing.com</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMi4gFBVV95cUxOUGt6RmJ4NjFGNHBKQUFnVXN4NVlIZzU3aEx1VkRwU3pSbVhUZWdEZEljX0JFR3ZhU3JvQUdma0ZsaS1LeW1TU0NPOUozazE2NHFxMjBhcmZPZnhYVHotVzM1VzRFWHBvWFR3LUV3YVRrOEpxSEJxSXdWVTZpQ3J6aUZwQjNJU2pjbVZwZWF4Z2c0SkdEM0N6WDE1S01LWjBpNWtvb3A4ZmFqRmlBTGRyQ3dxU0czelNZcEZ4U3RoRFdMSFZmT1d4Q2pvc3VUU2FLTElkUUNpaU91Vlp4Z0lBSDZB?oc=5</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T02:37:57+00:00</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="n"/>
+      <c r="I63" s="2" t="n"/>
+      <c r="J63" s="2" t="n"/>
+      <c r="K63" s="2" t="n"/>
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>AI agents</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Godfather of AI Yann LeCun does not believe that AI will kill humans; 'blames' humans for AI Agents hacki - The Times of India</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>The Times of India</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgNBVV95cUxOazNWRGJLVlVMbXpWeV9VRUp5bU83QnVuOTdlcG1ORFlKZXZ2NkdadW9fNTNZQkJLVDJpaDFsU1hGSDJtdlFrNVMzYVlFZ0ZTWXVyeEcwTnZwczJmRVlKSDBzZGNSN1hRV2gxUWFZYUp6UWNrU21LOUdWdVBvQ2tuVGZQXzdPeXQ3MDNEblEzd1Bab0hOb0VZWXNYWHdBVE1IdnBpVWN4UUtrMFBYZDZ5d1NOa3c3MEhGREN5MGJCY3U5STE0ZGt1LWlHdHVkZk1mM3VCSDFFZndlalpLcEFfY0RiT3lkM01hUUFjNmotcFE5aUpHNFgzbEV4OW9leGp1c2xULVFaY1p6QXIwdE9rUS1yYXdzRnRtMmMyVlBRcThFdWhTSkl5SVVNLUd5OXlvanJwLTVWR2FkRm10d2NXYTdIcVZRa19DY2NwLWpjRzhqN2h6LVRjcGZqWTBOenpsR2Q5VXpBMlFFcXk4VVpnMTc0dVNyNkhZczBnZzZLYThJVmxwTVlXbWZ2NEg3QdIBkwNBVV95cUxNVFdmUk5BWjBjbU5aVkpsd1BzMi1Wd3BXRmtMU1lTTUwxTUVJRlcydTNJWGROV1l3Y1hCLXpzbGlzUDlQY0tFNG56S0JsaGQ2SnY5azVqRXdBbHg2b2x4a2lWWmNuQnZuRUw1LXBBVHpvZnBjZ1hkVDZDYkVnbVRMOHR5aTd0dGZVZGx4ZGE0ekVHNERwbUxuS3NYZEFSZlh2ZmZYRFFOZFlRdTIzMU5jQkdMdU9fNWdaeFcwTl9RMkE5eTR3M1ZPQlFUTTd1eGpjTzhqajJUb0xRR3hIMkRXdUdZN0dIcURJbEwzLWxoODJjb3NxUUJFLURXXy00ZEhuLTJldDdSSVd0c093eGhzbkJhTzc4emF0OU9xQ2ZBb2RZejlLcHZtT3pXTzV6cUVncmxfX1MtVmFBdWFpd05ZSVZldXVXby16a0NoUXJJTU41WnV5WXpLa0RNVnlSN1Qzdm9qandHRGs3OU82ZmZtZURiMElPM2R0d0NaN2tHN21UWGI5QUltZ0EtTkUyTEFrNVBV?oc=5</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T06:24:00+00:00</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="n"/>
+      <c r="I64" s="2" t="n"/>
+      <c r="J64" s="2" t="n"/>
+      <c r="K64" s="2" t="n"/>
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N64" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>AI agents</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>When AI agents slip the leash: How companies monitor and control them - The Indian Express</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>The Indian Express</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipwFBVV95cUxOWE5IaXkzdTRtZmJLcXZVMWw5Zk9Hb2JjQUlPYVlFQmJFcHNwRS1PZnhpaTlRWk15Q1hYX2FkY091RURtOHNmQWVYR1VURVdNZDZqVjdtd0htSmYxYzhGTzR6RGpRanpEOUg1VC01UmNLSkdIa0ZDVXUtSHB3SWJhZVRLeDNsR2hWV1pKdHBEVUVNWlA0Y213M1JJTEFlUlI4SjZreXUtNNIBrgFBVV95cUxNTUh5YlBuYUoyNmFoNVJZa3RqbzlSR3ZRamFQU2RGbDRpZHdLdzdocnBCa1JPNkNmWGRrR3JLNEJvdzZWdXM0U1diWVBGVnNpMmd1WUk2ano2ZDhaOG56cjVLVEhjcGIyMC1Dd2lWcEVwRDZ0cGotdktXQk1VczdyUWhLZXFEaldDbFlfakR4eGFqdWpoby1Ncl9CQnpqa2VMZmRLTlZoODdmQ2l5NXc?oc=5</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T08:17:03+00:00</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="n"/>
+      <c r="I65" s="2" t="n"/>
+      <c r="J65" s="2" t="n"/>
+      <c r="K65" s="2" t="n"/>
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N65" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>AI agents</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Consumer AI agents: What does it mean for Financial Services? By Investing.com - Investing.com India</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Investing.com India</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMirwFBVV95cUxPaU9vU011OE1PdDNoMzRpMzlOdW82OEdpNVZVbGk3M3pmMHRRZmxJdE1oTWVQY0tpR0F0SEtIR1hBQUFkaGVzMl9xN1pTN1NURDJMRGItSXZ1Y1lMVVVxWUd0SEZXbEVTN1lrdkxLcm1vWWl3cUNyeTk3SEhOQVBOYk1jZGhybi1jOWl4LTJ1dW9qNjlQajcwTWV1ZHhueVEtNHg0aE5DQUg1UWRLRmVn?oc=5</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T08:17:24+00:00</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="n"/>
+      <c r="I66" s="2" t="n"/>
+      <c r="J66" s="2" t="n"/>
+      <c r="K66" s="2" t="n"/>
+      <c r="L66" s="2" t="n"/>
+      <c r="M66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N66" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>AI agents</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Who’s to Blame When A.I. Goes Rogue? - The New York Times</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>The New York Times</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiggFBVV95cUxQTUhrakN2TGFTTmdhM0VtY2s5UjBjOVB5cnRRM1NHOWxPV1FGYTdfYjRrQkNZeFFBeHVkSXI1Q29DOE96WmNnSndCb1hwU1c4UGpxanNmMlJsNkJkYVRZNEpBSzdLdG55cXN5Z3hBYWVZSVVkQ1B2OV81Q1hEbExJUUJR?oc=5</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:51:00+00:00</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="n"/>
+      <c r="I67" s="2" t="n"/>
+      <c r="J67" s="2" t="n"/>
+      <c r="K67" s="2" t="n"/>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>AI coding tools</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>3 years in software job, but cannot explain his own code: AI is killing 'critical thinking' skills even am - The Economic Times</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>The Economic Times</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqwJBVV95cUxPcXNBWDRaRmlDNG53ZFBhTmlqSS1LUDlSaVFzSmhXNzNFWXFTZm5RdGhpNVF0anY4ZGtwSVNVUTlsbW51YXRudmNBR2JxdzNNeERtYjB5VEwyTDB0TlBCOVhEMUNpUUhYU1VuT2VybC1waWFFTWdIdHhfODMwWkhFZldaaVpwNzJSWThDNFhtdFZNek44UU16UWVsUm1hZGVyWnVSY2RIdFlRMnNoc1VXNFFMUk9IWlVKeGI0UTAzLWI4eFVnVk55ZHZfQk1FVEtMSWhKVi1URDZ6RzZJZHRMeC1VTVQzZnNndUZLc2FpWUY3T3lwblowaVQwYnVNQkF1UWVXZ1lFUEtQSk5OUi1oVHpiTEZ0RG5CQkpKbjlvRnh0QS1uNHA2VUNtUdIBsAJBVV95cUxQSUhoT09KTk5wZDN6amp0b3dRbDlfSmVEYmFOODJoSHBVV2N0cDg5UENDaW5yWEh3MGpNUGd3N0pxUmRneUJ0TkkyS1pJck1qMmNzWUUteTc0dVNXQmo0ZWhtb1R2SnBMS3NCb1ZURVgtei1SQWhENlBONDRfZjJCYlNaZGNtdFlBZ205WXM3NVFJbjRUMXZPQ0R0TUVXei1KZU12ay1ERHBWVmdheGdvbXJyS1hpa3FvTnE2NHBVbVFUOGwxOWZMdVg2SksxRmo4RG5JaFJ5bzJHX1ExMElpR3hKbWdmdUw0LTdKTUJiR1Z4RTVBNlVkbGdraUc3dkM4eEY4dnZXdXJ1TGxaUGptRWF0bV9CVExSdU5TLUtfR0xlU3NMRTc5TUxYNVZ0aHk4?oc=5</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:47:28+00:00</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="n"/>
+      <c r="I68" s="2" t="n"/>
+      <c r="J68" s="2" t="n"/>
+      <c r="K68" s="2" t="n"/>
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N68" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>open source AI</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Meta launches open source Muse Gadgets project for custom AI hardware - Indian Television Dot Com</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Indian Television Dot Com</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMiqgFBVV95cUxPV2tuN1NMVjdTMEJDRHE1bnFMV2JhaVF6bDEtTDlwLTlPTk5xMVVZejFYTGZHU05uTFNGaFNYem9iWk0yNnVLcy1WZHoxVTlBRnFOOVJJSG5xMVRRN0Q5S3FKOFNuTi1jYmpOUzZvbUJHeEFBbzJ3RVFUMUV1Y2NadGF6WElzRDV0aUxYRlhwQTZLeTJHRTJBd1ZzVllOX0h1c1M1QUpxNHM5dw?oc=5</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T14:40:36+00:00</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="n"/>
+      <c r="I69" s="2" t="n"/>
+      <c r="J69" s="2" t="n"/>
+      <c r="K69" s="2" t="n"/>
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N69" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>news</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>robotics AI</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>From Surgery to Diagnostics: Robotics Enters New Healthcare Frontiers - The Indian Practitioner</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>The Indian Practitioner</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMipgFBVV95cUxOWl9WbmUwMmNYc21SMkZNT3lhY2x3d2hxS2FWQjVaMEJWVG52R1NsZ1FHTE01ZUpVRkMzcl9MaE1rZG9TeG5ocURkb0Z3bGR2RGQzUGpoTzBCN25zbEx3S2RqYkxBRS1mWUNPeXpvb01MMEZlWmpvWXhiY0NUUEpyYkl6VnFzdkhpamg1cl9VVzBzUWNyUFNuaHVoM2FFVlhaekJXU29n?oc=5</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03T12:09:15+00:00</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="n"/>
+      <c r="I70" s="2" t="n"/>
+      <c r="J70" s="2" t="n"/>
+      <c r="K70" s="2" t="n"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>researched</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:O1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3140,7 +4200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3279,6 +4339,88 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Apple limiting AI agents full disk access on Mac</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>మీ Mac డేటాపై AI నిఘా? Apple సంచలన నిర్ణయం!</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>మీ కంప్యూటర్‌లోని మొత్తం డేటాను AI ఏజెంట్లు సైలెంట్‌గా చూసేస్తున్నాయా?</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>See research.json and source links</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPUDRRTmRHQURXblJFVlgwQ2JpNUFLRVVBcTNRVmxKRDgzX1pWbVUxZHJfeUNBTlVsT0pQV2Q5T2xOdzFjQ1FlQ09NajFXU2xfODhBNVNiOWJIbnphRTF2VDJzNWEtTHBpOFlGSmw5Tmtnc2FUcjBKTVExeDZ6MFNlSFh2ODlYWmh4OFZtb1FR?oc=5
+https://news.google.com/rss/articles/CBMilAFBVV95cUxQSS1DeTVFM3prNm9wck9fNTczNnEwcFFyaUs5eFpDZ0QzN1NDMDdtelVpYWR3YUx0cWZKMkpLRmFsYmJnQXhDblNiNU9kSFNRNGZ2ZTMyZXBKZU9kbVZnV29NakhyNGFZX3FfTWZlZTJhTmJkRGhJcmhNbjVTbno3YlNnRTFNU2FTcm1DcVFKckFhRFp2?oc=5</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Apple limiting AI agents full disk access on Mac</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>మీ Mac డేటాపై AI నిఘా? Apple సంచలన నిర్ణయం!</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>మీ కంప్యూటర్‌లోని మొత్తం డేటాను AI ఏజెంట్లు సైలెంట్‌గా చూసేస్తున్నాయా?</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>See research.json and source links</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://news.google.com/rss/articles/CBMijgFBVV95cUxPUDRRTmRHQURXblJFVlgwQ2JpNUFLRVVBcTNRVmxKRDgzX1pWbVUxZHJfeUNBTlVsT0pQV2Q5T2xOdzFjQ1FlQ09NajFXU2xfODhBNVNiOWJIbnphRTF2VDJzNWEtTHBpOFlGSmw5Tmtnc2FUcjBKTVExeDZ6MFNlSFh2ODlYWmh4OFZtb1FR?oc=5
+https://news.google.com/rss/articles/CBMilAFBVV95cUxQSS1DeTVFM3prNm9wck9fNTczNnEwcFFyaUs5eFpDZ0QzN1NDMDdtelVpYWR3YUx0cWZKMkpLRmFsYmJnQXhDblNiNU9kSFNRNGZ2ZTMyZXBKZU9kbVZnV29NakhyNGFZX3FfTWZlZTJhTmJkRGhJcmhNbjVTbno3YlNnRTFNU2FTcm1DcVFKckFhRFp2?oc=5</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>selected</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3291,7 +4433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3414,6 +4556,80 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>మీ Mac డేటాపై AI నిఘా? Apple సంచలన నిర్ణయం!</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>మీ కంప్యూటర్‌లోని మొత్తం డేటాను AI ఏజెంట్లు సైలెంట్‌గా చూసేస్తున్నాయా? దీనికి అడ్డుకట్ట వేయడానికి Apple ఇప్పుడు ఒక పెద్ద నిర్ణయం తీసుకుంది! సాధారణ చాట్‌బాట్ల కంటే భిన్నంగా, మన కంప్యూటర్‌లో సొంతంగా పనులు పూర్తి చేసే అటానమస్ AI agents ఇప్పుడు ట్రెండ్ అవుతున్నాయి. అయితే కొన్ని AI టూల్స్ మన సిస్టమ్‌లోని ఫుల్ డిస్క్ యాక్సెస్ పర్మిషన్స్ తీసుకుంటున్నట్లు టెక్ నిపుణులు హెచ్చరిస్తున్నారు. ఒకసారి ఫుల్ యాక్సెస్ వస్తే, మీ ప్రైవేట్ ఫైల్స్, బ్రౌజింగ్ డేటా, చివరికి కీలక సమాచారం కూడా వాటి చేతుల్లోకి వెళ్లే ప్రమాదం ఉంది. అందుకే Mac కంప్యూటర్లలో ఇలాంటి రిస్క్‌లకు బ్రేక్ వేసేందుకు Apple కొత్త భద్రతా నిబంధనలను సిద్ధం చేస్తోంది. రాబోయే అప్‌డేట్‌తో, ఏ AI ఏజెంట్‌ కూడా యూజర్ స్పష్టమైన అనుమతి లేకుండా డిస్క్‌లోని ఫైళ్లను టచ్ చేయలేదు. ఆర్టిఫిషియల్ ఇంటెలిజెన్స్ ఎంత వేగంగా ఎదుగుతోందో, సైబర్ సెక్యూరిటీ రక్షణలు కూడా అంతే కఠినంగా మారాల్సిన అవసరం ఏర్పడింది. టెక్నాలజీ ఇచ్చే సౌలభ్యాన్ని ఆస్వాదించండి, కానీ ఏ యాప్‌కైనా పర్మిషన్లు ఇచ్చే ముందు ఎల్లప్పుడూ జాగ్రత్తగా పరిశీలించండి!</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>A slick 9:16 vertical short about AI agent security on Apple MacBooks. Fast-paced camera zooms on a sleek MacBook displaying neon security shield graphics, illuminated digital lock icons over folder trees, and dynamic motion graphics showing AI autonomous processes. High contrast cyber aesthetics, clean Telugu typography overlays, smooth split-screen animations, soft cinematic background synth hum, crisp Telugu voiceover, clear burned-in subtitles, and a definitive takeaway card at the end.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Mac యూజర్ల డేటా భద్రత కోసం Apple కీలక అడుగు వేస్తోంది. AI ఏజెంట్లకు ఫుల్ డిస్క్ యాక్సెస్ పరిమితులపై తాజా వివరాలు తెలుసుకోండి! #Apple #AI #Mac #TechNews #TeluguTech</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>#AI #Apple #Technology #తెలుగు #TechNewsTelugu</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>rendered</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>మీ Mac డేటాపై AI నిఘా? Apple సంచలన నిర్ణయం!</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>మీ కంప్యూటర్‌లోని మొత్తం డేటాను AI ఏజెంట్లు సైలెంట్‌గా చూసేస్తున్నాయా? దీనికి అడ్డుకట్ట వేయడానికి Apple ఇప్పుడు ఒక పెద్ద నిర్ణయం తీసుకుంది! సాధారణ చాట్‌బాట్ల కంటే భిన్నంగా, మన కంప్యూటర్‌లో సొంతంగా పనులు పూర్తి చేసే అటానమస్ AI agents ఇప్పుడు ట్రెండ్ అవుతున్నాయి. అయితే కొన్ని AI టూల్స్ మన సిస్టమ్‌లోని ఫుల్ డిస్క్ యాక్సెస్ పర్మిషన్స్ తీసుకుంటున్నట్లు టెక్ నిపుణులు హెచ్చరిస్తున్నారు. ఒకసారి ఫుల్ యాక్సెస్ వస్తే, మీ ప్రైవేట్ ఫైల్స్, బ్రౌజింగ్ డేటా, చివరికి కీలక సమాచారం కూడా వాటి చేతుల్లోకి వెళ్లే ప్రమాదం ఉంది. అందుకే Mac కంప్యూటర్లలో ఇలాంటి రిస్క్‌లకు బ్రేక్ వేసేందుకు Apple కొత్త భద్రతా నిబంధనలను సిద్ధం చేస్తోంది. రాబోయే అప్‌డేట్‌తో, ఏ AI ఏజెంట్‌ కూడా యూజర్ స్పష్టమైన అనుమతి లేకుండా డిస్క్‌లోని ఫైళ్లను టచ్ చేయలేదు. ఆర్టిఫిషియల్ ఇంటెలిజెన్స్ ఎంత వేగంగా ఎదుగుతోందో, సైబర్ సెక్యూరిటీ రక్షణలు కూడా అంతే కఠినంగా మారాల్సిన అవసరం ఏర్పడింది. టెక్నాలజీ ఇచ్చే సౌలభ్యాన్ని ఆస్వాదించండి, కానీ ఏ యాప్‌కైనా పర్మిషన్లు ఇచ్చే ముందు ఎల్లప్పుడూ జాగ్రత్తగా పరిశీలించండి!</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>A slick 9:16 vertical short about AI agent security on Apple MacBooks. Fast-paced camera zooms on a sleek MacBook displaying neon security shield graphics, illuminated digital lock icons over folder trees, and dynamic motion graphics showing AI autonomous processes. High contrast cyber aesthetics, clean Telugu typography overlays, smooth split-screen animations, soft cinematic background synth hum, crisp Telugu voiceover, clear burned-in subtitles, and a definitive takeaway card at the end.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Mac యూజర్ల డేటా భద్రత కోసం Apple కీలక అడుగు వేస్తోంది. AI ఏజెంట్లకు ఫుల్ డిస్క్ యాక్సెస్ పరిమితులపై తాజా వివరాలు తెలుసుకోండి! #Apple #AI #Mac #TechNews #TeluguTech</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>#AI #Apple #Technology #తెలుగు #TechNewsTelugu</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>rendered</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3426,7 +4642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3490,6 +4706,33 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>మీ Mac డేటాపై AI నిఘా? Apple సంచలన నిర్ణయం!</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>8JHYTqy-kAk</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=8JHYTqy-kAk</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>uploaded</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>